<commit_message>
Updated topics and links
</commit_message>
<xml_diff>
--- a/Learning Time Frame.xlsx
+++ b/Learning Time Frame.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="138">
   <si>
     <t>Topic ID</t>
   </si>
@@ -113,10 +113,19 @@
     <t>VectorDB</t>
   </si>
   <si>
+    <t>https://docs.google.com/document/d/1Gc97w2TCsJDd698NqsmyQ9Kua3qR03b0lgYIqxHfn_8/edit?usp=sharing</t>
+  </si>
+  <si>
+    <t>AWS Lambda &amp; SQS</t>
+  </si>
+  <si>
+    <t>Cloud</t>
+  </si>
+  <si>
     <t>In Progress</t>
   </si>
   <si>
-    <t>https://docs.google.com/document/d/1Gc97w2TCsJDd698NqsmyQ9Kua3qR03b0lgYIqxHfn_8/edit?usp=sharing</t>
+    <t>https://docs.google.com/document/d/1N-fcqICz1tOX27XlgKzBlrvEAcUpOiArtTp4TnsfO34/edit?usp=sharing</t>
   </si>
   <si>
     <t>Sub Topic ID</t>
@@ -329,9 +338,6 @@
     <t>Indexing and Performance</t>
   </si>
   <si>
-    <t>Not Started</t>
-  </si>
-  <si>
     <t>Hybrid Search</t>
   </si>
   <si>
@@ -339,6 +345,45 @@
   </si>
   <si>
     <t>Advanced APIs</t>
+  </si>
+  <si>
+    <t>AWS Lambda Fundamentals - Serverless concepts, Lambda architecture, runtimes, handlers, deployment packages, environment variables</t>
+  </si>
+  <si>
+    <t>Not Started</t>
+  </si>
+  <si>
+    <t>Lambda Execution Model - Invocation lifecycle, cold starts, warm starts, memory allocation, CPU allocation, timeouts, execution environment reuse</t>
+  </si>
+  <si>
+    <t>Lambda Triggers &amp; Event Sources - API Gateway, S3, EventBridge, DynamoDB Streams, SQS triggers</t>
+  </si>
+  <si>
+    <t>Lambda Security &amp; Monitoring - IAM roles, execution roles, CloudWatch Logs, Metrics, X-Ray</t>
+  </si>
+  <si>
+    <t>Lambda Error Handling &amp; Optimization - Retries, DLQ, destinations, concurrency, provisioned concurrency, cost optimization</t>
+  </si>
+  <si>
+    <t>Amazon SQS Fundamentals - Message queues, async communication, producer-consumer pattern, queue architecture</t>
+  </si>
+  <si>
+    <t>SQS Queue Types &amp; Message Lifecycle - Standard vs FIFO, ordering, deduplication, send/receive/delete flow, retention period</t>
+  </si>
+  <si>
+    <t>SQS Advanced Concepts - Visibility timeout, long polling, short polling, message attributes, encryption, monitoring</t>
+  </si>
+  <si>
+    <t>Dead Letter Queues (DLQ) - Redrive policies, failed message processing, troubleshooting</t>
+  </si>
+  <si>
+    <t>Lambda + SQS Integration - Event source mapping, polling, batching, scaling, concurrency</t>
+  </si>
+  <si>
+    <t>Failure Handling in Lambda + SQS - Retries, poison messages, partial batch failures, DLQ integration</t>
+  </si>
+  <si>
+    <t>Monitoring &amp; Production Readiness - CloudWatch dashboards, alarms, troubleshooting, logging strategy</t>
   </si>
   <si>
     <t>tool</t>
@@ -368,7 +413,7 @@
     <t>Memory</t>
   </si>
   <si>
-    <t>Pinecone, weaviate, qdrant,FAISS</t>
+    <t>Pinecone, weaviate,FAISS</t>
   </si>
   <si>
     <t>bokeh viz</t>
@@ -639,7 +684,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I9" displayName="Main_Topics" name="Main_Topics" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I10" displayName="Main_Topics" name="Main_Topics" id="1">
   <tableColumns count="9">
     <tableColumn name="Topic ID" id="1"/>
     <tableColumn name="Topic" id="2"/>
@@ -656,7 +701,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I64" displayName="Table1" name="Table1" id="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I76" displayName="Table1" name="Table1" id="2">
   <tableColumns count="9">
     <tableColumn name="Sub Topic ID" id="1"/>
     <tableColumn name="Sub-Topics" id="2"/>
@@ -1159,23 +1204,45 @@
       <c r="E9" s="12">
         <v>46097.0</v>
       </c>
-      <c r="F9" s="12"/>
+      <c r="F9" s="12">
+        <v>46094.0</v>
+      </c>
       <c r="G9" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="H9" s="15" t="s">
         <v>32</v>
-      </c>
-      <c r="H9" s="15" t="s">
-        <v>33</v>
       </c>
       <c r="I9" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="5"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="I10" s="5"/>
+    <row r="10" ht="22.5" customHeight="1">
+      <c r="A10" s="10">
+        <v>9000.0</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" s="12">
+        <v>46191.0</v>
+      </c>
+      <c r="E10" s="12">
+        <v>46209.0</v>
+      </c>
+      <c r="F10" s="12"/>
+      <c r="G10" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="H10" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5"/>
@@ -8116,7 +8183,7 @@
     </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G2:G9">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G2:G10">
       <formula1>"Not Started,In Progress,Completed,Paused"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8137,10 +8204,12 @@
     <hyperlink display="GO" location="'Sub Topics'!A50" ref="I8"/>
     <hyperlink r:id="rId8" ref="H9"/>
     <hyperlink display="GO" location="'Sub Topics'!A59" ref="I9"/>
+    <hyperlink r:id="rId9" ref="H10"/>
+    <hyperlink display="GO" location="'Sub Topics'!A65" ref="I10"/>
   </hyperlinks>
-  <drawing r:id="rId9"/>
+  <drawing r:id="rId10"/>
   <tableParts count="1">
-    <tablePart r:id="rId11"/>
+    <tablePart r:id="rId12"/>
   </tableParts>
 </worksheet>
 </file>
@@ -8165,19 +8234,19 @@
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
       <c r="A1" s="18" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F1" s="18" t="s">
         <v>4</v>
@@ -8186,10 +8255,10 @@
         <v>5</v>
       </c>
       <c r="H1" s="18" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="I1" s="18" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="J1" s="20"/>
       <c r="K1" s="20"/>
@@ -8204,7 +8273,7 @@
         <v>1001.0</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C2" s="23" t="s">
         <v>9</v>
@@ -8225,7 +8294,7 @@
         <v>11</v>
       </c>
       <c r="I2" s="22" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="J2" s="25"/>
       <c r="K2" s="25"/>
@@ -8240,7 +8309,7 @@
         <v>1002.0</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C3" s="23" t="s">
         <v>9</v>
@@ -8261,7 +8330,7 @@
         <v>11</v>
       </c>
       <c r="I3" s="22" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="J3" s="25"/>
       <c r="K3" s="25"/>
@@ -8276,7 +8345,7 @@
         <v>1003.0</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C4" s="23" t="s">
         <v>9</v>
@@ -8297,7 +8366,7 @@
         <v>11</v>
       </c>
       <c r="I4" s="22" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="J4" s="25"/>
       <c r="K4" s="25"/>
@@ -8312,7 +8381,7 @@
         <v>1004.0</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C5" s="23" t="s">
         <v>9</v>
@@ -8333,7 +8402,7 @@
         <v>11</v>
       </c>
       <c r="I5" s="22" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="J5" s="25"/>
       <c r="K5" s="25"/>
@@ -8348,7 +8417,7 @@
         <v>2001.0</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>14</v>
@@ -8369,7 +8438,7 @@
         <v>11</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
@@ -8377,7 +8446,7 @@
         <v>2002.0</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>14</v>
@@ -8404,7 +8473,7 @@
         <v>2003.0</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>14</v>
@@ -8425,7 +8494,7 @@
         <v>11</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
@@ -8433,7 +8502,7 @@
         <v>3001.0</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>16</v>
@@ -8454,7 +8523,7 @@
         <v>11</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
@@ -8462,7 +8531,7 @@
         <v>3002.0</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>16</v>
@@ -8483,7 +8552,7 @@
         <v>11</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
@@ -8491,7 +8560,7 @@
         <v>3003.0</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>16</v>
@@ -8512,7 +8581,7 @@
         <v>11</v>
       </c>
       <c r="I11" s="11" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
@@ -8520,7 +8589,7 @@
         <v>3004.0</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>16</v>
@@ -8541,7 +8610,7 @@
         <v>11</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
@@ -8549,7 +8618,7 @@
         <v>3005.0</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>16</v>
@@ -8570,7 +8639,7 @@
         <v>11</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
@@ -8578,7 +8647,7 @@
         <v>3006.0</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>16</v>
@@ -8599,7 +8668,7 @@
         <v>11</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" ht="22.5" customHeight="1">
@@ -8607,7 +8676,7 @@
         <v>3007.0</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>16</v>
@@ -8628,7 +8697,7 @@
         <v>11</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
@@ -8636,7 +8705,7 @@
         <v>3008.0</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>16</v>
@@ -8657,7 +8726,7 @@
         <v>11</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
@@ -8665,7 +8734,7 @@
         <v>3009.0</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>16</v>
@@ -8686,7 +8755,7 @@
         <v>11</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
@@ -8694,7 +8763,7 @@
         <v>4001.0</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>19</v>
@@ -8715,7 +8784,7 @@
         <v>11</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" ht="22.5" customHeight="1">
@@ -8723,7 +8792,7 @@
         <v>4002.0</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>19</v>
@@ -8744,7 +8813,7 @@
         <v>11</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" ht="22.5" customHeight="1">
@@ -8752,7 +8821,7 @@
         <v>4003.0</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>19</v>
@@ -8773,7 +8842,7 @@
         <v>11</v>
       </c>
       <c r="I20" s="11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="21" ht="22.5" customHeight="1">
@@ -8781,7 +8850,7 @@
         <v>4004.0</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>19</v>
@@ -8802,7 +8871,7 @@
         <v>11</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="22" ht="22.5" customHeight="1">
@@ -8810,7 +8879,7 @@
         <v>4005.0</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>19</v>
@@ -8831,7 +8900,7 @@
         <v>11</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="23" ht="22.5" customHeight="1">
@@ -8839,7 +8908,7 @@
         <v>4006.0</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C23" s="7" t="s">
         <v>19</v>
@@ -8860,7 +8929,7 @@
         <v>11</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24" ht="22.5" customHeight="1">
@@ -8868,7 +8937,7 @@
         <v>4007.0</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>19</v>
@@ -8889,7 +8958,7 @@
         <v>11</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25" ht="22.5" customHeight="1">
@@ -8897,7 +8966,7 @@
         <v>4008.0</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>19</v>
@@ -8918,7 +8987,7 @@
         <v>11</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" ht="22.5" customHeight="1">
@@ -8926,7 +8995,7 @@
         <v>4009.0</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>19</v>
@@ -8947,7 +9016,7 @@
         <v>11</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27" ht="22.5" customHeight="1">
@@ -8955,7 +9024,7 @@
         <v>4010.0</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>19</v>
@@ -8976,7 +9045,7 @@
         <v>11</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" ht="22.5" customHeight="1">
@@ -8984,7 +9053,7 @@
         <v>4011.0</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C28" s="7" t="s">
         <v>19</v>
@@ -9005,7 +9074,7 @@
         <v>11</v>
       </c>
       <c r="I28" s="11" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="29" ht="22.5" customHeight="1">
@@ -9013,7 +9082,7 @@
         <v>4012.0</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C29" s="7" t="s">
         <v>19</v>
@@ -9034,7 +9103,7 @@
         <v>11</v>
       </c>
       <c r="I29" s="11" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30" ht="22.5" customHeight="1">
@@ -9042,7 +9111,7 @@
         <v>4013.0</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C30" s="7" t="s">
         <v>19</v>
@@ -9063,7 +9132,7 @@
         <v>11</v>
       </c>
       <c r="I30" s="11" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="31" ht="22.5" customHeight="1">
@@ -9071,7 +9140,7 @@
         <v>5001.0</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C31" s="14" t="s">
         <v>22</v>
@@ -9092,7 +9161,7 @@
         <v>11</v>
       </c>
       <c r="I31" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32" ht="22.5" customHeight="1">
@@ -9100,7 +9169,7 @@
         <v>5002.0</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C32" s="14" t="s">
         <v>22</v>
@@ -9121,7 +9190,7 @@
         <v>11</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="33" ht="22.5" customHeight="1">
@@ -9129,7 +9198,7 @@
         <v>5003.0</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C33" s="14" t="s">
         <v>22</v>
@@ -9150,7 +9219,7 @@
         <v>11</v>
       </c>
       <c r="I33" s="11" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="34" ht="22.5" customHeight="1">
@@ -9158,7 +9227,7 @@
         <v>5004.0</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C34" s="14" t="s">
         <v>22</v>
@@ -9179,7 +9248,7 @@
         <v>11</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="35" ht="22.5" customHeight="1">
@@ -9187,7 +9256,7 @@
         <v>5005.0</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C35" s="14" t="s">
         <v>22</v>
@@ -9208,7 +9277,7 @@
         <v>11</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="36" ht="22.5" customHeight="1">
@@ -9216,7 +9285,7 @@
         <v>5006.0</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C36" s="14" t="s">
         <v>22</v>
@@ -9237,7 +9306,7 @@
         <v>11</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="37" ht="22.5" customHeight="1">
@@ -9245,7 +9314,7 @@
         <v>5007.0</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C37" s="14" t="s">
         <v>22</v>
@@ -9266,7 +9335,7 @@
         <v>11</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="38" ht="22.5" customHeight="1">
@@ -9274,7 +9343,7 @@
         <v>5008.0</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C38" s="14" t="s">
         <v>22</v>
@@ -9295,7 +9364,7 @@
         <v>11</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="39" ht="22.5" customHeight="1">
@@ -9303,7 +9372,7 @@
         <v>5009.0</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C39" s="14" t="s">
         <v>22</v>
@@ -9324,7 +9393,7 @@
         <v>11</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="40" ht="22.5" customHeight="1">
@@ -9332,7 +9401,7 @@
         <v>5010.0</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C40" s="14" t="s">
         <v>22</v>
@@ -9353,7 +9422,7 @@
         <v>11</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="41" ht="22.5" customHeight="1">
@@ -9361,7 +9430,7 @@
         <v>5011.0</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C41" s="14" t="s">
         <v>22</v>
@@ -9382,7 +9451,7 @@
         <v>11</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="42" ht="22.5" customHeight="1">
@@ -9390,7 +9459,7 @@
         <v>5012.0</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C42" s="14" t="s">
         <v>22</v>
@@ -9411,7 +9480,7 @@
         <v>11</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="43" ht="22.5" customHeight="1">
@@ -9419,7 +9488,7 @@
         <v>5013.0</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C43" s="14" t="s">
         <v>22</v>
@@ -9440,7 +9509,7 @@
         <v>11</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="44" ht="22.5" customHeight="1">
@@ -9448,7 +9517,7 @@
         <v>5014.0</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C44" s="14" t="s">
         <v>22</v>
@@ -9469,7 +9538,7 @@
         <v>11</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="45" ht="22.5" customHeight="1">
@@ -9477,7 +9546,7 @@
         <v>6001.0</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C45" s="14" t="s">
         <v>25</v>
@@ -9498,7 +9567,7 @@
         <v>11</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="46" ht="22.5" customHeight="1">
@@ -9506,7 +9575,7 @@
         <v>6002.0</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C46" s="14" t="s">
         <v>25</v>
@@ -9527,7 +9596,7 @@
         <v>11</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="47" ht="22.5" customHeight="1">
@@ -9535,7 +9604,7 @@
         <v>6003.0</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C47" s="14" t="s">
         <v>25</v>
@@ -9556,7 +9625,7 @@
         <v>11</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="48" ht="22.5" customHeight="1">
@@ -9564,7 +9633,7 @@
         <v>6004.0</v>
       </c>
       <c r="B48" s="11" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C48" s="14" t="s">
         <v>25</v>
@@ -9585,7 +9654,7 @@
         <v>11</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="49" ht="22.5" customHeight="1">
@@ -9593,7 +9662,7 @@
         <v>6005.0</v>
       </c>
       <c r="B49" s="11" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C49" s="14" t="s">
         <v>25</v>
@@ -9614,7 +9683,7 @@
         <v>11</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="50" ht="22.5" customHeight="1">
@@ -9622,7 +9691,7 @@
         <v>7001.0</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C50" s="14" t="s">
         <v>27</v>
@@ -9643,7 +9712,7 @@
         <v>11</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="51" ht="22.5" customHeight="1">
@@ -9651,7 +9720,7 @@
         <v>7002.0</v>
       </c>
       <c r="B51" s="11" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C51" s="14" t="s">
         <v>27</v>
@@ -9672,7 +9741,7 @@
         <v>11</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="52" ht="22.5" customHeight="1">
@@ -9680,7 +9749,7 @@
         <v>7003.0</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C52" s="14" t="s">
         <v>27</v>
@@ -9701,7 +9770,7 @@
         <v>11</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="53" ht="22.5" customHeight="1">
@@ -9709,7 +9778,7 @@
         <v>7004.0</v>
       </c>
       <c r="B53" s="11" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C53" s="14" t="s">
         <v>27</v>
@@ -9730,7 +9799,7 @@
         <v>11</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="54" ht="22.5" customHeight="1">
@@ -9738,7 +9807,7 @@
         <v>7005.0</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C54" s="14" t="s">
         <v>27</v>
@@ -9759,7 +9828,7 @@
         <v>11</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="55" ht="22.5" customHeight="1">
@@ -9767,7 +9836,7 @@
         <v>7006.0</v>
       </c>
       <c r="B55" s="11" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C55" s="14" t="s">
         <v>27</v>
@@ -9788,7 +9857,7 @@
         <v>11</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="56" ht="22.5" customHeight="1">
@@ -9796,7 +9865,7 @@
         <v>7007.0</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C56" s="14" t="s">
         <v>27</v>
@@ -9817,7 +9886,7 @@
         <v>11</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="57" ht="22.5" customHeight="1">
@@ -9825,7 +9894,7 @@
         <v>7008.0</v>
       </c>
       <c r="B57" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C57" s="14" t="s">
         <v>27</v>
@@ -9846,7 +9915,7 @@
         <v>11</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="58" ht="22.5" customHeight="1">
@@ -9854,7 +9923,7 @@
         <v>7009.0</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C58" s="14" t="s">
         <v>27</v>
@@ -9875,7 +9944,7 @@
         <v>11</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="59" ht="22.5" customHeight="1">
@@ -9883,7 +9952,7 @@
         <v>8001.0</v>
       </c>
       <c r="B59" s="11" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C59" s="14" t="s">
         <v>30</v>
@@ -9897,18 +9966,22 @@
       <c r="F59" s="12">
         <v>46086.0</v>
       </c>
-      <c r="G59" s="12"/>
+      <c r="G59" s="12">
+        <v>46086.0</v>
+      </c>
       <c r="H59" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="I59" s="11"/>
+      <c r="I59" s="11" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="60" ht="22.5" customHeight="1">
       <c r="A60" s="10">
         <v>8002.0</v>
       </c>
       <c r="B60" s="11" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C60" s="14" t="s">
         <v>30</v>
@@ -9922,18 +9995,22 @@
       <c r="F60" s="12">
         <v>46087.0</v>
       </c>
-      <c r="G60" s="12"/>
+      <c r="G60" s="12">
+        <v>46087.0</v>
+      </c>
       <c r="H60" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="I60" s="11"/>
+        <v>11</v>
+      </c>
+      <c r="I60" s="11" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="61" ht="22.5" customHeight="1">
       <c r="A61" s="10">
         <v>8003.0</v>
       </c>
       <c r="B61" s="11" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C61" s="14" t="s">
         <v>30</v>
@@ -9941,22 +10018,28 @@
       <c r="D61" s="12">
         <v>46090.0</v>
       </c>
-      <c r="E61" s="12"/>
+      <c r="E61" s="12">
+        <v>46090.0</v>
+      </c>
       <c r="F61" s="12">
         <v>46090.0</v>
       </c>
-      <c r="G61" s="12"/>
+      <c r="G61" s="12">
+        <v>46090.0</v>
+      </c>
       <c r="H61" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="I61" s="11"/>
+        <v>11</v>
+      </c>
+      <c r="I61" s="11" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="62" ht="22.5" customHeight="1">
       <c r="A62" s="10">
         <v>8004.0</v>
       </c>
       <c r="B62" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C62" s="14" t="s">
         <v>30</v>
@@ -9964,22 +10047,28 @@
       <c r="D62" s="12">
         <v>46091.0</v>
       </c>
-      <c r="E62" s="12"/>
+      <c r="E62" s="12">
+        <v>46091.0</v>
+      </c>
       <c r="F62" s="12">
         <v>46091.0</v>
       </c>
-      <c r="G62" s="12"/>
+      <c r="G62" s="12">
+        <v>46091.0</v>
+      </c>
       <c r="H62" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="I62" s="11"/>
+        <v>11</v>
+      </c>
+      <c r="I62" s="11" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="63" ht="22.5" customHeight="1">
       <c r="A63" s="10">
         <v>8005.0</v>
       </c>
       <c r="B63" s="11" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C63" s="14" t="s">
         <v>30</v>
@@ -9987,22 +10076,28 @@
       <c r="D63" s="12">
         <v>46092.0</v>
       </c>
-      <c r="E63" s="12"/>
+      <c r="E63" s="12">
+        <v>46092.0</v>
+      </c>
       <c r="F63" s="12">
         <v>46092.0</v>
       </c>
-      <c r="G63" s="12"/>
+      <c r="G63" s="12">
+        <v>46092.0</v>
+      </c>
       <c r="H63" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="I63" s="11"/>
+        <v>11</v>
+      </c>
+      <c r="I63" s="11" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="64" ht="22.5" customHeight="1">
       <c r="A64" s="10">
         <v>8006.0</v>
       </c>
       <c r="B64" s="11" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C64" s="14" t="s">
         <v>30</v>
@@ -10010,99 +10105,297 @@
       <c r="D64" s="12">
         <v>46093.0</v>
       </c>
-      <c r="E64" s="12"/>
+      <c r="E64" s="12">
+        <v>46093.0</v>
+      </c>
       <c r="F64" s="12">
         <v>46094.0</v>
       </c>
-      <c r="G64" s="12"/>
+      <c r="G64" s="12">
+        <v>46094.0</v>
+      </c>
       <c r="H64" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="I64" s="11"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="5"/>
-      <c r="D65" s="5"/>
-      <c r="E65" s="5"/>
-      <c r="F65" s="5"/>
-      <c r="G65" s="5"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="5"/>
-      <c r="D66" s="5"/>
-      <c r="E66" s="5"/>
-      <c r="F66" s="5"/>
-      <c r="G66" s="5"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="5"/>
-      <c r="D67" s="5"/>
-      <c r="E67" s="5"/>
-      <c r="F67" s="5"/>
-      <c r="G67" s="5"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="5"/>
-      <c r="D68" s="5"/>
-      <c r="E68" s="5"/>
-      <c r="F68" s="5"/>
-      <c r="G68" s="5"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="5"/>
-      <c r="D69" s="5"/>
-      <c r="E69" s="5"/>
-      <c r="F69" s="5"/>
-      <c r="G69" s="5"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="5"/>
-      <c r="D70" s="5"/>
-      <c r="E70" s="5"/>
-      <c r="F70" s="5"/>
-      <c r="G70" s="5"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="5"/>
-      <c r="D71" s="5"/>
-      <c r="E71" s="5"/>
-      <c r="F71" s="5"/>
-      <c r="G71" s="5"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="5"/>
-      <c r="D72" s="5"/>
-      <c r="E72" s="5"/>
-      <c r="F72" s="5"/>
-      <c r="G72" s="5"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="5"/>
-      <c r="D73" s="5"/>
-      <c r="E73" s="5"/>
-      <c r="F73" s="5"/>
-      <c r="G73" s="5"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="5"/>
-      <c r="D74" s="5"/>
-      <c r="E74" s="5"/>
-      <c r="F74" s="5"/>
-      <c r="G74" s="5"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="5"/>
-      <c r="D75" s="5"/>
-      <c r="E75" s="5"/>
-      <c r="F75" s="5"/>
-      <c r="G75" s="5"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="5"/>
-      <c r="D76" s="5"/>
-      <c r="E76" s="5"/>
-      <c r="F76" s="5"/>
-      <c r="G76" s="5"/>
+        <v>11</v>
+      </c>
+      <c r="I64" s="11" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="65" ht="22.5" customHeight="1">
+      <c r="A65" s="10">
+        <v>9001.0</v>
+      </c>
+      <c r="B65" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="C65" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D65" s="12">
+        <v>46191.0</v>
+      </c>
+      <c r="E65" s="12"/>
+      <c r="F65" s="12">
+        <v>46191.0</v>
+      </c>
+      <c r="G65" s="12"/>
+      <c r="H65" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="I65" s="11"/>
+    </row>
+    <row r="66" ht="22.5" customHeight="1">
+      <c r="A66" s="10">
+        <v>9002.0</v>
+      </c>
+      <c r="B66" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="C66" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D66" s="12">
+        <v>46192.0</v>
+      </c>
+      <c r="E66" s="12"/>
+      <c r="F66" s="12">
+        <v>46192.0</v>
+      </c>
+      <c r="G66" s="12"/>
+      <c r="H66" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="I66" s="11"/>
+    </row>
+    <row r="67" ht="22.5" customHeight="1">
+      <c r="A67" s="10">
+        <v>9003.0</v>
+      </c>
+      <c r="B67" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="C67" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D67" s="12">
+        <v>46195.0</v>
+      </c>
+      <c r="E67" s="12"/>
+      <c r="F67" s="12">
+        <v>46195.0</v>
+      </c>
+      <c r="G67" s="12"/>
+      <c r="H67" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="I67" s="11"/>
+    </row>
+    <row r="68" ht="22.5" customHeight="1">
+      <c r="A68" s="10">
+        <v>9004.0</v>
+      </c>
+      <c r="B68" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="C68" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D68" s="12">
+        <v>46196.0</v>
+      </c>
+      <c r="E68" s="12"/>
+      <c r="F68" s="12">
+        <v>46196.0</v>
+      </c>
+      <c r="G68" s="12"/>
+      <c r="H68" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="I68" s="11"/>
+    </row>
+    <row r="69" ht="22.5" customHeight="1">
+      <c r="A69" s="10">
+        <v>9005.0</v>
+      </c>
+      <c r="B69" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="C69" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D69" s="12">
+        <v>46197.0</v>
+      </c>
+      <c r="E69" s="12"/>
+      <c r="F69" s="12">
+        <v>46197.0</v>
+      </c>
+      <c r="G69" s="12"/>
+      <c r="H69" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="I69" s="11"/>
+    </row>
+    <row r="70" ht="22.5" customHeight="1">
+      <c r="A70" s="10">
+        <v>9006.0</v>
+      </c>
+      <c r="B70" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="C70" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D70" s="12">
+        <v>46198.0</v>
+      </c>
+      <c r="E70" s="12"/>
+      <c r="F70" s="12">
+        <v>46198.0</v>
+      </c>
+      <c r="G70" s="12"/>
+      <c r="H70" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="I70" s="11"/>
+    </row>
+    <row r="71" ht="22.5" customHeight="1">
+      <c r="A71" s="10">
+        <v>9007.0</v>
+      </c>
+      <c r="B71" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="C71" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D71" s="12">
+        <v>46199.0</v>
+      </c>
+      <c r="E71" s="12"/>
+      <c r="F71" s="12">
+        <v>46199.0</v>
+      </c>
+      <c r="G71" s="12"/>
+      <c r="H71" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="I71" s="11"/>
+    </row>
+    <row r="72" ht="22.5" customHeight="1">
+      <c r="A72" s="10">
+        <v>9008.0</v>
+      </c>
+      <c r="B72" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="C72" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D72" s="12">
+        <v>46202.0</v>
+      </c>
+      <c r="E72" s="12"/>
+      <c r="F72" s="12">
+        <v>46202.0</v>
+      </c>
+      <c r="G72" s="12"/>
+      <c r="H72" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="I72" s="11"/>
+    </row>
+    <row r="73" ht="22.5" customHeight="1">
+      <c r="A73" s="10">
+        <v>9009.0</v>
+      </c>
+      <c r="B73" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="C73" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D73" s="12">
+        <v>46203.0</v>
+      </c>
+      <c r="E73" s="12"/>
+      <c r="F73" s="12">
+        <v>46203.0</v>
+      </c>
+      <c r="G73" s="12"/>
+      <c r="H73" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="I73" s="11"/>
+    </row>
+    <row r="74" ht="22.5" customHeight="1">
+      <c r="A74" s="10">
+        <v>9010.0</v>
+      </c>
+      <c r="B74" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="C74" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D74" s="12">
+        <v>46204.0</v>
+      </c>
+      <c r="E74" s="12"/>
+      <c r="F74" s="12">
+        <v>46205.0</v>
+      </c>
+      <c r="G74" s="12"/>
+      <c r="H74" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="I74" s="11"/>
+    </row>
+    <row r="75" ht="22.5" customHeight="1">
+      <c r="A75" s="10">
+        <v>9011.0</v>
+      </c>
+      <c r="B75" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="C75" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D75" s="12">
+        <v>46206.0</v>
+      </c>
+      <c r="E75" s="12"/>
+      <c r="F75" s="12">
+        <v>46206.0</v>
+      </c>
+      <c r="G75" s="12"/>
+      <c r="H75" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="I75" s="11"/>
+    </row>
+    <row r="76" ht="22.5" customHeight="1">
+      <c r="A76" s="10">
+        <v>9012.0</v>
+      </c>
+      <c r="B76" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="C76" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D76" s="12">
+        <v>46209.0</v>
+      </c>
+      <c r="E76" s="12"/>
+      <c r="F76" s="12">
+        <v>46209.0</v>
+      </c>
+      <c r="G76" s="12"/>
+      <c r="H76" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="I76" s="11"/>
     </row>
     <row r="77">
       <c r="A77" s="5"/>
@@ -16567,16 +16860,16 @@
     </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="E2:G64">
+    <dataValidation type="list" allowBlank="1" sqref="C2:C76">
+      <formula1>#REF!</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="E2:G76">
       <formula1>OR(NOT(ISERROR(DATEVALUE(E2))), AND(ISNUMBER(E2), LEFT(CELL("format", E2))="D"))</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C2:C64">
-      <formula1>#REF!</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H2:H64">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H2:H76">
       <formula1>"Not Started,In Progress,Completed,Paused"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I2:I64">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I2:I76">
       <formula1>"YouTube,ChatGPT,Web"</formula1>
     </dataValidation>
   </dataValidations>
@@ -16601,59 +16894,59 @@
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
       <c r="A1" s="26" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="D2" s="27" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="D3" s="27" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="D4" s="27" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="6" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>121</v>
+        <v>136</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>122</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>

</xml_diff>